<commit_message>
Final Version of the board
</commit_message>
<xml_diff>
--- a/parts_list.xlsx
+++ b/parts_list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\KjB22\Desktop\Kicad Projects\ENGT481\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A59B8924-4128-4390-9DCE-04405076FC0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C2158DF-EA74-4510-9534-28E4215803D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{EC1EF8A6-F3C8-49CE-B7CB-3A00316C7F8D}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="62">
   <si>
     <t>USB4500-03-1-A</t>
   </si>
@@ -65,12 +65,6 @@
     <t>BQ24040DSQR</t>
   </si>
   <si>
-    <t>STM32</t>
-  </si>
-  <si>
-    <t>STM32WB55CGUx</t>
-  </si>
-  <si>
     <t>EXB-28V103JX</t>
   </si>
   <si>
@@ -134,12 +128,6 @@
     <t>SOD-123 schottky diode</t>
   </si>
   <si>
-    <t>0402 Ferrite Bead</t>
-  </si>
-  <si>
-    <t>BLM15AG601SN1D</t>
-  </si>
-  <si>
     <t>DSS14U</t>
   </si>
   <si>
@@ -231,6 +219,9 @@
   </si>
   <si>
     <t>STM32 MCU</t>
+  </si>
+  <si>
+    <t>PCB</t>
   </si>
 </sst>
 </file>
@@ -261,12 +252,18 @@
       <name val="Roboto"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -281,18 +278,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -637,321 +636,324 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="C2" t="s">
+      <c r="B2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+    </row>
+    <row r="4" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D4" s="2">
+        <v>1578</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+    </row>
+    <row r="6" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B8" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="E8" s="8"/>
+    </row>
+    <row r="9" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B9" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="E9" s="8"/>
+    </row>
+    <row r="10" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B10" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B11" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B12" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="D13" s="1"/>
+    </row>
+    <row r="14" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B14" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B15" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B16" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B17" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="18" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B18" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D18" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="D2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B4" t="s">
+    </row>
+    <row r="20" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B20" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="21" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B21" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="22" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B22" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="23" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B23" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="24" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B24" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="26" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B26" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C4" t="s">
-        <v>55</v>
-      </c>
-      <c r="D4">
-        <v>1578</v>
-      </c>
-    </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B6" t="s">
-        <v>26</v>
-      </c>
-      <c r="C6" t="s">
-        <v>64</v>
-      </c>
-      <c r="D6" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B8" t="s">
-        <v>26</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="E8" s="6"/>
-    </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C9" s="2" t="s">
+      <c r="D26" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="28" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B28" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C28" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D9" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="E9" s="6"/>
-    </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B10" t="s">
-        <v>26</v>
-      </c>
-      <c r="C10" t="s">
-        <v>3</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B11" t="s">
-        <v>26</v>
-      </c>
-      <c r="C11" t="s">
-        <v>5</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B12" t="s">
-        <v>26</v>
-      </c>
-      <c r="C12" t="s">
-        <v>7</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C13" t="s">
-        <v>9</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B14" t="s">
-        <v>26</v>
-      </c>
-      <c r="C14" t="s">
-        <v>12</v>
-      </c>
-      <c r="D14" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B15" t="s">
-        <v>18</v>
-      </c>
-      <c r="C15" t="s">
-        <v>13</v>
-      </c>
-      <c r="D15" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B16" t="s">
-        <v>26</v>
-      </c>
-      <c r="C16" t="s">
-        <v>15</v>
-      </c>
-      <c r="D16" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B17" t="s">
-        <v>26</v>
-      </c>
-      <c r="C17" t="s">
+      <c r="D28" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="30" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B30" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D30" s="2"/>
+    </row>
+    <row r="32" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B32" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="34" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B34" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="35" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B35" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="36" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B36" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="37" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B37" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="38" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B38" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C38" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D38" s="2" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B18" t="s">
-        <v>26</v>
-      </c>
-      <c r="C18" t="s">
-        <v>51</v>
-      </c>
-      <c r="D18" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B20" t="s">
-        <v>18</v>
-      </c>
-      <c r="C20" t="s">
-        <v>17</v>
-      </c>
-      <c r="D20" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B21" t="s">
-        <v>19</v>
-      </c>
-      <c r="C21" t="s">
-        <v>20</v>
-      </c>
-      <c r="D21" t="s">
+    <row r="40" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B40" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C40" s="2" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="22" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B22" t="s">
-        <v>22</v>
-      </c>
-      <c r="C22" t="s">
-        <v>21</v>
-      </c>
-      <c r="D22" t="s">
+      <c r="D40" s="7" t="s">
         <v>58</v>
-      </c>
-    </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B23" t="s">
-        <v>19</v>
-      </c>
-      <c r="C23" t="s">
-        <v>23</v>
-      </c>
-      <c r="D23" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="24" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B24" t="s">
-        <v>24</v>
-      </c>
-      <c r="C24" t="s">
-        <v>25</v>
-      </c>
-      <c r="D24" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="26" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B26" t="s">
-        <v>26</v>
-      </c>
-      <c r="C26" t="s">
-        <v>28</v>
-      </c>
-      <c r="D26" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="28" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B28" t="s">
-        <v>30</v>
-      </c>
-      <c r="C28" t="s">
-        <v>31</v>
-      </c>
-      <c r="D28" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="30" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B30" t="s">
-        <v>26</v>
-      </c>
-      <c r="C30" t="s">
-        <v>32</v>
-      </c>
-      <c r="D30" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="32" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B32" t="s">
-        <v>19</v>
-      </c>
-      <c r="C32" t="s">
-        <v>46</v>
-      </c>
-      <c r="D32" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="34" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B34" t="s">
-        <v>37</v>
-      </c>
-      <c r="C34" t="s">
-        <v>35</v>
-      </c>
-      <c r="D34" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="35" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B35" t="s">
-        <v>30</v>
-      </c>
-      <c r="C35" t="s">
-        <v>38</v>
-      </c>
-      <c r="D35" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="36" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B36" t="s">
-        <v>37</v>
-      </c>
-      <c r="C36" t="s">
-        <v>40</v>
-      </c>
-      <c r="D36" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="37" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B37" t="s">
-        <v>42</v>
-      </c>
-      <c r="C37" t="s">
-        <v>43</v>
-      </c>
-      <c r="D37" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="38" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B38" t="s">
-        <v>37</v>
-      </c>
-      <c r="C38" t="s">
-        <v>53</v>
-      </c>
-      <c r="D38" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="40" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B40" t="s">
-        <v>26</v>
-      </c>
-      <c r="C40" t="s">
-        <v>61</v>
-      </c>
-      <c r="D40" s="5" t="s">
-        <v>62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>